<commit_message>
Added new RDF data schemes and visual schemes for employment-table22-23, fixed XLSX spreadsheets for employment-table22-23
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/employment-table22.xlsx
+++ b/sources/table_normalization/xlsx/employment-table22.xlsx
@@ -161,13 +161,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -474,15 +474,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
@@ -490,49 +490,49 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="4">
         <v>2023</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="7"/>
-      <c r="B5" s="6" t="s">
+      <c r="A5" s="5"/>
+      <c r="B5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6" t="s">
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
     </row>
     <row r="6" spans="1:7" ht="57" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="7"/>
-      <c r="B6" s="3" t="s">
+      <c r="A6" s="5"/>
+      <c r="B6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="7" t="s">
         <v>7</v>
       </c>
     </row>
@@ -951,15 +951,15 @@
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" s="5" t="s">
+      <c r="A30" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B30" s="5"/>
-      <c r="C30" s="5"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
-      <c r="G30" s="5"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>